<commit_message>
Update ranker with score normalization and update submission files
</commit_message>
<xml_diff>
--- a/prompts_pirates.xlsx
+++ b/prompts_pirates.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>444.6361</v>
+        <v>0.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -466,7 +466,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>436.4815</v>
+        <v>0.9454</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -484,7 +484,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>423.2584</v>
+        <v>0.873</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -502,7 +502,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>421.7245</v>
+        <v>0.8646</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>415.1498</v>
+        <v>0.8286</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -538,7 +538,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>409.9054</v>
+        <v>0.7999000000000001</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -556,7 +556,7 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>407.9183</v>
+        <v>0.789</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>406.2437</v>
+        <v>0.7798</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>403.4313</v>
+        <v>0.7644</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>402.5606</v>
+        <v>0.7597</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -628,7 +628,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>399.8446</v>
+        <v>0.7448</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>397.5431</v>
+        <v>0.7322</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>395.804</v>
+        <v>0.7227</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>385.3668</v>
+        <v>0.6655</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>383.6321</v>
+        <v>0.656</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>380.4858</v>
+        <v>0.6388</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -736,7 +736,7 @@
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>379.4822</v>
+        <v>0.6333</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>376.0246</v>
+        <v>0.6143999999999999</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>371.2417</v>
+        <v>0.5881999999999999</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>367.6834</v>
+        <v>0.5687</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -808,7 +808,7 @@
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>367.4772</v>
+        <v>0.5676</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>367.3288</v>
+        <v>0.5668</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>365.5209</v>
+        <v>0.5569</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>364.6931</v>
+        <v>0.5523</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>360.4837</v>
+        <v>0.5293</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>355.6655</v>
+        <v>0.5029</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>351.1212</v>
+        <v>0.478</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -934,7 +934,7 @@
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>350.3812</v>
+        <v>0.474</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -952,7 +952,7 @@
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>347.1802</v>
+        <v>0.4565</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>346.3203</v>
+        <v>0.4518</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -988,7 +988,7 @@
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>345.1862</v>
+        <v>0.4456</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>344.8818</v>
+        <v>0.4439</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>343.4699</v>
+        <v>0.4362</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1042,7 +1042,7 @@
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>342.4275</v>
+        <v>0.4304</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>342.3155</v>
+        <v>0.4298</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1078,7 +1078,7 @@
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>342.2835</v>
+        <v>0.4297</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1096,7 +1096,7 @@
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>341.8414</v>
+        <v>0.4272</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1114,7 +1114,7 @@
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>341.3005</v>
+        <v>0.4243</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1132,7 +1132,7 @@
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>341.1465</v>
+        <v>0.4234</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>340.8299</v>
+        <v>0.4217</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1168,7 +1168,7 @@
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>339.896</v>
+        <v>0.4166</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>339.1286</v>
+        <v>0.4124</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1204,7 +1204,7 @@
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>339.0294</v>
+        <v>0.4118</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1222,7 +1222,7 @@
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>337.3543</v>
+        <v>0.4027</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1240,7 +1240,7 @@
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>336.1683</v>
+        <v>0.3962</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>335.6255</v>
+        <v>0.3932</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>334.8335</v>
+        <v>0.3889</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1294,7 +1294,7 @@
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>334.2746</v>
+        <v>0.3858</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>333.3889</v>
+        <v>0.381</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1330,7 +1330,7 @@
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>333.0841</v>
+        <v>0.3793</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>332.8789</v>
+        <v>0.3782</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1366,7 +1366,7 @@
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>331.6602</v>
+        <v>0.3715</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1384,7 +1384,7 @@
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>331.0922</v>
+        <v>0.3684</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1402,7 +1402,7 @@
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>329.5773</v>
+        <v>0.3601</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1420,7 +1420,7 @@
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>328.7938</v>
+        <v>0.3558</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>326.8392</v>
+        <v>0.3451</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1456,7 +1456,7 @@
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>326.4848</v>
+        <v>0.3432</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>324.8691</v>
+        <v>0.3343</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>324.6082</v>
+        <v>0.3329</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>324.5654</v>
+        <v>0.3327</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>323.8573</v>
+        <v>0.3288</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1546,7 +1546,7 @@
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>323.6279</v>
+        <v>0.3275</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1564,7 +1564,7 @@
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>323.4796</v>
+        <v>0.3267</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>322.8629</v>
+        <v>0.3233</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -1600,7 +1600,7 @@
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>322.1749</v>
+        <v>0.3196</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>322.1124</v>
+        <v>0.3192</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>321.3197</v>
+        <v>0.3149</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>321.2573</v>
+        <v>0.3145</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -1672,7 +1672,7 @@
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>319.8006</v>
+        <v>0.3066</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>318.7018</v>
+        <v>0.3006</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>316.2444</v>
+        <v>0.2871</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1726,7 +1726,7 @@
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>316.0441</v>
+        <v>0.286</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1744,7 +1744,7 @@
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>315.0623</v>
+        <v>0.2806</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -1762,7 +1762,7 @@
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>314.7763</v>
+        <v>0.2791</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>314.1701</v>
+        <v>0.2758</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>314.0973</v>
+        <v>0.2754</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>312.0593</v>
+        <v>0.2642</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>310.8137</v>
+        <v>0.2574</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>310.7821</v>
+        <v>0.2572</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>310.7162</v>
+        <v>0.2568</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>310.4151</v>
+        <v>0.2552</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>310.3976</v>
+        <v>0.2551</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -1924,7 +1924,7 @@
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>309.5578</v>
+        <v>0.2505</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>308.6929</v>
+        <v>0.2458</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -1960,7 +1960,7 @@
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>307.762</v>
+        <v>0.2407</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -1978,7 +1978,7 @@
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>307.2368</v>
+        <v>0.2378</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -1996,7 +1996,7 @@
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>306.674</v>
+        <v>0.2347</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>306.3865</v>
+        <v>0.2331</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>306.248</v>
+        <v>0.2324</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -2050,7 +2050,7 @@
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>306.0747</v>
+        <v>0.2314</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2068,7 +2068,7 @@
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>304.531</v>
+        <v>0.223</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2086,7 +2086,7 @@
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>304.1128</v>
+        <v>0.2207</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>303.865</v>
+        <v>0.2193</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2122,7 +2122,7 @@
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>303.5385</v>
+        <v>0.2175</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2140,7 +2140,7 @@
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>301.9508</v>
+        <v>0.2089</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>301.7824</v>
+        <v>0.2079</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2176,7 +2176,7 @@
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>300.8238</v>
+        <v>0.2027</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -2194,7 +2194,7 @@
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>300.7139</v>
+        <v>0.2021</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2212,7 +2212,7 @@
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>300.6669</v>
+        <v>0.2018</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -2230,7 +2230,7 @@
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>300.3335</v>
+        <v>0.2</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>

</xml_diff>